<commit_message>
Move capa/autoridades/comissao para a planilha; remove coluna obrigatorio
Frontmatter (capa, autoridades, comissao de elaboracao) deixa de vir de
YAML separado e passa a ser lido de novas abas/campos da propria
matriz_curricular.xlsx, unificando tudo num so lugar. Coluna
obrigatorio da aba Componentes eh removida: obrigatorio passa a ser
derivado de tipo != carga_optativa, eliminando a divergencia possivel
entre os dois campos.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testes/perfis_exemplo/matriz_curricular.xlsx
+++ b/testes/perfis_exemplo/matriz_curricular.xlsx
@@ -972,7 +972,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:M5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1003,45 +1003,40 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>obrigatorio</t>
+          <t>cht</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>cht</t>
+          <t>chp</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>chp</t>
+          <t>chd</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>chd</t>
+          <t>che</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>che</t>
+          <t>tot</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>tot</t>
+          <t>observacoes</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>observacoes</t>
+          <t>pre_requisitos</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
-        <is>
-          <t>pre_requisitos</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
         <is>
           <t>correquisitos</t>
         </is>
@@ -1069,11 +1064,11 @@
       <c r="E2" t="b">
         <v>1</v>
       </c>
-      <c r="F2" t="b">
-        <v>1</v>
+      <c r="F2" t="n">
+        <v>30</v>
       </c>
       <c r="G2" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1082,9 +1077,6 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
         <v>30</v>
       </c>
     </row>
@@ -1110,11 +1102,11 @@
       <c r="E3" t="b">
         <v>1</v>
       </c>
-      <c r="F3" t="b">
-        <v>1</v>
+      <c r="F3" t="n">
+        <v>30</v>
       </c>
       <c r="G3" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -1123,12 +1115,9 @@
         <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
         <v>30</v>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>D1</t>
         </is>
@@ -1156,8 +1145,8 @@
       <c r="E4" t="b">
         <v>1</v>
       </c>
-      <c r="F4" t="b">
-        <v>1</v>
+      <c r="F4" t="n">
+        <v>0</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -1166,14 +1155,11 @@
         <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="J4" t="n">
         <v>15</v>
       </c>
-      <c r="K4" t="n">
-        <v>15</v>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1194,11 +1180,11 @@
       <c r="E5" t="b">
         <v>1</v>
       </c>
-      <c r="F5" t="b">
+      <c r="F5" t="n">
+        <v>30</v>
+      </c>
+      <c r="G5" t="n">
         <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>30</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -1207,9 +1193,6 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
         <v>30</v>
       </c>
     </row>

</xml_diff>

<commit_message>
gerando a segunda versão
</commit_message>
<xml_diff>
--- a/testes/perfis_exemplo/matriz_curricular.xlsx
+++ b/testes/perfis_exemplo/matriz_curricular.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:B48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -693,155 +693,155 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>curriculo.carga_optativa_minima</t>
+          <t>curriculo.carga_extensao</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>curriculo.carga_extensao</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>15</v>
+          <t>curriculo.carga_aac</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>curriculo.carga_aac</t>
+          <t>curriculo.carga_estagio</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>curriculo.carga_estagio</t>
+          <t>curriculo.carga_tcc</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>curriculo.carga_tcc</t>
+          <t>curriculo.percentual_minimo_extensao</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>curriculo.percentual_minimo_extensao</t>
+          <t>curriculo.percentual_maximo_ead</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>curriculo.percentual_maximo_ead</t>
+          <t>curriculo.carga_horaria_presencial_maxima_periodo</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>curriculo.carga_horaria_presencial_maxima_periodo</t>
+          <t>curriculo.periodo_minimo_tcc</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>curriculo.periodo_minimo_tcc</t>
+          <t>curriculo.periodo_minimo_estagio</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>curriculo.periodo_minimo_estagio</t>
+          <t>arquivos.textos</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>textos</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>arquivos.textos</t>
+          <t>arquivos.fichas</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>textos</t>
+          <t>fichas</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>arquivos.fichas</t>
+          <t>arquivos.figuras</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>fichas</t>
+          <t>figuras</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>arquivos.figuras</t>
+          <t>arquivos.anexos</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>figuras</t>
+          <t>anexos</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>arquivos.anexos</t>
+          <t>arquivos.overrides</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>anexos</t>
+          <t>overrides</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>arquivos.overrides</t>
+          <t>geracao.template</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>overrides</t>
+          <t>padrao</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>geracao.template</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>padrao</t>
-        </is>
+          <t>geracao.anexar_fichas</t>
+        </is>
+      </c>
+      <c r="B39" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>geracao.anexar_fichas</t>
+          <t>geracao.anexar_resolucoes</t>
         </is>
       </c>
       <c r="B40" t="b">
@@ -851,7 +851,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>geracao.anexar_resolucoes</t>
+          <t>geracao.gerar_fluxo_curricular</t>
         </is>
       </c>
       <c r="B41" t="b">
@@ -861,7 +861,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>geracao.gerar_fluxo_curricular</t>
+          <t>geracao.gerar_representacao_grafica</t>
         </is>
       </c>
       <c r="B42" t="b">
@@ -871,7 +871,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>geracao.gerar_representacao_grafica</t>
+          <t>geracao.gerar_relatorio_validacao</t>
         </is>
       </c>
       <c r="B43" t="b">
@@ -881,7 +881,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>geracao.gerar_relatorio_validacao</t>
+          <t>geracao.compilar_pdf</t>
         </is>
       </c>
       <c r="B44" t="b">
@@ -891,7 +891,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>geracao.compilar_pdf</t>
+          <t>geracao.interromper_em_erro</t>
         </is>
       </c>
       <c r="B45" t="b">
@@ -901,42 +901,32 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>geracao.interromper_em_erro</t>
-        </is>
-      </c>
-      <c r="B46" t="b">
-        <v>1</v>
+          <t>saida.nome_base</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>PPC_perfil_minimo</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>saida.nome_base</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>PPC_perfil_minimo</t>
-        </is>
+          <t>saida.gerar_corpo</t>
+        </is>
+      </c>
+      <c r="B47" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>saida.gerar_corpo</t>
+          <t>saida.gerar_completo</t>
         </is>
       </c>
       <c r="B48" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>saida.gerar_completo</t>
-        </is>
-      </c>
-      <c r="B49" t="b">
         <v>1</v>
       </c>
     </row>
@@ -972,7 +962,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1193,6 +1183,41 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>MODOPT</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MÓDULO OPTATIVO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>carga_optativa</t>
+        </is>
+      </c>
+      <c r="E6" t="b">
+        <v>0</v>
+      </c>
+      <c r="F6" t="n">
+        <v>30</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" t="n">
         <v>30</v>
       </c>
     </row>

</xml_diff>